<commit_message>
Fixed Redemption and Reward Menu Test Cases Failure
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/02_ClaimPoints/ClaimPoints/04_ClaimInformationPageTest.xlsx
+++ b/src/test/resources/testdata/Modules/02_ClaimPoints/ClaimPoints/04_ClaimInformationPageTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\02_ClaimPoints\ClaimPoints\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01269EA0-1E00-49A4-8388-704DCEF0F792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A7FD917-CB26-441E-8C76-F2BBC2FFF47B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="91">
   <si>
     <t>TESTCASE_ID</t>
   </si>
@@ -877,12 +877,6 @@
 verify_warningmsg</t>
   </si>
   <si>
-    <t>claiminfo_enter_customermobileno
-hidekeyboard
-claiminfo_clikon_submitbtn
-verify_warningmsg</t>
-  </si>
-  <si>
     <t>Please enter valid mobile number</t>
   </si>
   <si>
@@ -892,23 +886,7 @@
     <t>select or capture all mandatory material Photos</t>
   </si>
   <si>
-    <t>claiminfo_clikon_materialproductimageicon
-clickonbrowsefileoption
-selectimageclickonbrowsefileoption
-claiminfo_clikon_submitbtn
-verify_warningmsg</t>
-  </si>
-  <si>
     <t>Please enter site address</t>
-  </si>
-  <si>
-    <t>Mayur colony, kothrud, Pune 411038</t>
-  </si>
-  <si>
-    <t>claiminfo_enter_siteaddress
-hidekeyboard
-claiminfo_clikon_submitbtn
-verify_warningmsg</t>
   </si>
   <si>
     <t>Please select or capture site photo</t>
@@ -1075,6 +1053,28 @@
 clickonbackarrow
 dealerlist_clickoncrossicon
 navigatebacktodashboardpage</t>
+  </si>
+  <si>
+    <t>waitforsnackbardisappear
+claiminfo_enter_customermobileno
+hidekeyboard
+claiminfo_clikon_submitbtn
+verify_warningmsg</t>
+  </si>
+  <si>
+    <t>waitforsnackbardisappear
+claiminfo_clikon_materialproductimageicon
+clickonbrowsefileoption
+selectimageclickonbrowsefileoption
+claiminfo_clikon_submitbtn
+verify_warningmsg</t>
+  </si>
+  <si>
+    <t>waitforsnackbardisappear
+claiminfo_enter_siteaddress
+hidekeyboard
+claiminfo_clikon_submitbtn
+verify_warningmsg</t>
   </si>
 </sst>
 </file>
@@ -2139,7 +2139,7 @@
         <v>23</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>38</v>
@@ -2179,7 +2179,7 @@
         <v>44</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>32</v>
@@ -2217,7 +2217,7 @@
         <v>48</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>38</v>
@@ -2257,7 +2257,7 @@
         <v>45</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>32</v>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
@@ -2297,7 +2297,7 @@
         <v>46</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>38</v>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
@@ -2337,7 +2337,7 @@
         <v>52</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>38</v>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
@@ -2377,7 +2377,7 @@
         <v>51</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>64</v>
@@ -2417,7 +2417,7 @@
         <v>54</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>38</v>
@@ -2475,7 +2475,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
@@ -2489,7 +2489,7 @@
         <v>56</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
@@ -2503,13 +2503,13 @@
       </c>
       <c r="N12" s="1"/>
       <c r="O12" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P12" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
@@ -2523,7 +2523,7 @@
         <v>57</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
@@ -2533,17 +2533,17 @@
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="N13" s="1"/>
       <c r="O13" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P13" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" ht="87" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>21</v>
       </c>
@@ -2557,7 +2557,7 @@
         <v>58</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
@@ -2569,13 +2569,13 @@
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="P14" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -2589,7 +2589,7 @@
         <v>59</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
@@ -2600,10 +2600,10 @@
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
       <c r="N15" s="1" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="P15" s="1" t="s">
         <v>5</v>
@@ -2623,7 +2623,7 @@
         <v>60</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
@@ -2776,7 +2776,7 @@
         <v>23</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>38</v>
@@ -2816,7 +2816,7 @@
         <v>44</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>32</v>
@@ -2854,7 +2854,7 @@
         <v>48</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>38</v>
@@ -2894,7 +2894,7 @@
         <v>45</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>32</v>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
@@ -2934,7 +2934,7 @@
         <v>46</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>38</v>
@@ -2948,7 +2948,7 @@
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
@@ -2974,7 +2974,7 @@
         <v>52</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>38</v>
@@ -2988,7 +2988,7 @@
       </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
@@ -3014,7 +3014,7 @@
         <v>51</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>64</v>
@@ -3054,7 +3054,7 @@
         <v>54</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>38</v>
@@ -3112,7 +3112,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
@@ -3126,7 +3126,7 @@
         <v>56</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
@@ -3140,13 +3140,13 @@
       </c>
       <c r="N12" s="1"/>
       <c r="O12" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P12" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
@@ -3160,7 +3160,7 @@
         <v>57</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
@@ -3170,17 +3170,17 @@
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="N13" s="1"/>
       <c r="O13" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P13" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" ht="87" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>21</v>
       </c>
@@ -3194,7 +3194,7 @@
         <v>58</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
@@ -3206,13 +3206,13 @@
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="P14" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -3226,7 +3226,7 @@
         <v>59</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
@@ -3237,10 +3237,10 @@
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
       <c r="N15" s="1" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="P15" s="1" t="s">
         <v>5</v>
@@ -3260,7 +3260,7 @@
         <v>60</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>

</xml_diff>

<commit_message>
Claim Module Failed Test Cases Update
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/02_ClaimPoints/ClaimPoints/04_ClaimInformationPageTest.xlsx
+++ b/src/test/resources/testdata/Modules/02_ClaimPoints/ClaimPoints/04_ClaimInformationPageTest.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\02_ClaimPoints\ClaimPoints\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E1FAEFC-8B51-4FD7-B721-1CE49DE2CF6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F8012AC-053E-4FA8-B755-7AD5F8CBB7BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="96">
   <si>
     <t>TESTCASE_ID</t>
   </si>
@@ -1144,6 +1144,27 @@
       </rPr>
       <t xml:space="preserve"> (non mandatory fo appium TMT)</t>
     </r>
+  </si>
+  <si>
+    <t>claiminfo_clikon_cancelbtn
+cartdetails_clickon_cancelbtn
+cartdetails_clickon_alertbox_yesbtn
+category_clickon_refreshbtn
+category_selectcategory
+category_selectbrand
+category_enterqty
+hidekeyboard
+category_select_product_diameter
+hidekeyboard
+category_clickon_addtocart_btn
+category_clickon_addtocart_btn
+category_clickon_carticon
+cartdetails_clickon_submitbtn
+claiminfo_clikon_submitbtn
+verify_warningmsg</t>
+  </si>
+  <si>
+    <t>Customer Name,Customer Mobile No</t>
   </si>
 </sst>
 </file>
@@ -2462,7 +2483,7 @@
         <v>88</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>57</v>
@@ -2475,7 +2496,9 @@
         <v>39</v>
       </c>
       <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
+      <c r="K9" s="9" t="s">
+        <v>95</v>
+      </c>
       <c r="L9" s="9"/>
       <c r="M9" s="9"/>
       <c r="N9" s="9"/>
@@ -2500,7 +2523,7 @@
         <v>48</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>36</v>

</xml_diff>